<commit_message>
Fix tracking-pack rebuild: keep a single UL-0005 row and freeze the instrument ID in Word.
Co-authored-by: delano2x-Procedurals <delano2x-Procedurals@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/Dissertation_Document_Tracking_Master.xlsx
+++ b/downloads/Dissertation_Document_Tracking_Master.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4068,470 +4068,939 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="48" customHeight="1">
-      <c r="A51" s="6" t="inlineStr">
+    <row r="51" ht="36" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>REF-WOOD-2021</t>
         </is>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>seminal_theory</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>build_on</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>Wood, D. J., Mitchell, R. K., Agle, B. R., &amp; Bryan, L. M. (2021). Stakeholder identification and salience after 20 years: Progress, problems, and prospects. Business &amp; Society, 60(1), 196–245. https://doi.org/10.1177/0007650318816522</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>Chapter II current review of salience research; does not replace Mitchell 1997 operational defs</t>
         </is>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>Spoken questions; theme titles; replacing Mitchell 1997</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H51" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
+      <c r="I51" s="5" t="inlineStr">
         <is>
           <t>03_REFERENCES</t>
         </is>
       </c>
-      <c r="J51" s="6" t="inlineStr">
+      <c r="J51" s="5" t="inlineStr">
         <is>
           <t>ITDR-GQI-INT-v0.1.1</t>
         </is>
       </c>
-      <c r="K51" s="6" t="inlineStr">
+      <c r="K51" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="L51" s="6" t="inlineStr">
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>Already in the GQI nest. Seminal/build-on rules unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="36" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>REF-JOOS-2019</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>seminal_theory</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>build_on</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Joos, H. C. (2019). Influences on managerial perceptions of stakeholder salience: Two decades of research in review. Management Review Quarterly, 69, 3–37. https://doi.org/10.1007/s11301-018-0144-8</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>What We Know: inner/outer context that shapes how managers perceive PLU. Sensitizing only.</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>Replacing Mitchell 1997; adding personality variables as codebook parents; findings</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>Wk3 PDF 8044-8927_Wk3_Influences_on_managerial_perce</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="M52" s="4" t="inlineStr">
+        <is>
+          <t>Already in the GQI nest. Seminal/build-on rules unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="36" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>REF-KHURRAM-2015</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>seminal_theory</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>build_on</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Khurram, S., &amp; Charreire Petit, S. (2017). Investigating the dynamics of stakeholder salience: What happens when the institutional change process unfolds? Journal of Business Ethics, 143(4), 663–680. https://doi.org/10.1007/s10551-015-2766-2</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>What We Know: salience attributes can shift as institutional logic shifts. Supports mid-incident C2 probes.</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>Study design (this is not an institutional-change case of microfinance); theme titles</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Wk10 PDF Investigating the Dynamics of Stakeholder Salience</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>Already in the GQI nest. Seminal/build-on rules unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="36" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>REF-EMR-ROADMAP-2023</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>seminal_method</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>build_on</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>verify</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Editorial. (2023). A roadmap for data analysis in qualitative research. European Management Review, 20(2), 190–196. (Duplicate course PDF of the same editorial; authors/page run EM-RAUS230022 — confirm named editorial authors before courseroom paste.)</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Know Eisenhardt / Gioia / Langley templates so they can be refused as this study’s method</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>Declaring Gioia, Eisenhardt, or Langley as the analytic method; replacing Fereday &amp; Muir-Cochrane 2006</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>Wk8 duplicate editorials</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>Already in the GQI nest. Seminal/build-on rules unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="36" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>REF-DANIEL-2019</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>comparative</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>build_on</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Daniel, E., &amp; Daniel, P. A. (2019). Megaprojects as complex adaptive systems: The Hinkley Point C case. International Journal of Project Management, 37(8), 1017–1033. https://doi.org/10.1016/j.ijproman.2019.05.001</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Parking lot / comparative complexity talk only</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>Design; sampling; coding system; Chapter IV themes; replacing GQI</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>Wk8 Hinkley Point C PDF</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>Already in the GQI nest. Seminal/build-on rules unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="36" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>REF-CHRISTENSEN-2023</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>comparative</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>build_on</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>Christensen, G. (2024). Three concepts of power: Foucault, Bourdieu, and Habermas. Power and Education, 16(2), 182–195. https://doi.org/10.1177/17577438231187129</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Optional P-memo language only after a concrete force/withhold/override example exists</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>Replacing Mitchell power; Delve parent codes; interview stems; educational-theory redesign</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>christensen-2023 PDF</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>parked</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>Already in the GQI nest. Seminal/build-on rules unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="36" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>REF-TRACKING-PACK-2026</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>audit_artifact</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>audit_artifact</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Walker, M. (2026). Dissertation document tracking pack (Pack v1.0) [Unpublished research operating file]. Capella University, RSCH-V8927. downloads/Dissertation_Document_Tracking_Master.xlsx; downloads/Dissertation_Document_Tracking_Pack.docx.</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Document control; change log; work schedule; folder map</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>Literature source; findings</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>this pack</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>Already in the GQI nest. Seminal/build-on rules unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="48" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>REF-WOOD-2021</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>seminal_theory</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>build_on</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Wood, D. J., Mitchell, R. K., Agle, B. R., &amp; Bryan, L. M. (2021). Stakeholder identification and salience after 20 years: Progress, problems, and prospects. Business &amp; Society, 60(1), 196–245. https://doi.org/10.1177/0007650318816522</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>Chapter II current review of salience research; does not replace Mitchell 1997 operational defs</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>Spoken questions; theme titles; replacing Mitchell 1997</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>03_REFERENCES</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="K58" s="6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L58" s="6" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="M51" s="6" t="inlineStr">
+      <c r="M58" s="6" t="inlineStr">
         <is>
           <t>Currency review requested in updated-references.md. Added as additional build-on, not as a swap that deletes Agle 1999 from the codebook nest.</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="48" customHeight="1">
-      <c r="A52" s="6" t="inlineStr">
+    <row r="59" ht="48" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>REF-JOOS-2019</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>seminal_theory</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>build_on</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>Joos, H. C. (2019). Influences on managerial perceptions of stakeholder salience: Two decades of research in review. Management Review Quarterly, 69, 3–37. https://doi.org/10.1007/s11301-018-0144-8</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>What We Know: inner/outer context that shapes how managers perceive PLU. Sensitizing only.</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>Replacing Mitchell 1997; adding personality variables as codebook parents; findings</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
+      <c r="I59" s="6" t="inlineStr">
         <is>
           <t>Wk3 PDF 8044-8927_Wk3_Influences_on_managerial_perce</t>
         </is>
       </c>
-      <c r="J52" s="6" t="inlineStr">
+      <c r="J59" s="6" t="inlineStr">
         <is>
           <t>ITDR-GQI-INT-v0.1.1</t>
         </is>
       </c>
-      <c r="K52" s="6" t="inlineStr">
+      <c r="K59" s="6" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="L52" s="6" t="inlineStr">
+      <c r="L59" s="6" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="M52" s="6" t="inlineStr">
+      <c r="M59" s="6" t="inlineStr">
         <is>
           <t>Course PDF now registered. Review of contextual influences; not a new salience attribute.</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="48" customHeight="1">
-      <c r="A53" s="6" t="inlineStr">
+    <row r="60" ht="48" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>REF-KHURRAM-2015</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>seminal_theory</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>build_on</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>Khurram, S., &amp; Charreire Petit, S. (2017). Investigating the dynamics of stakeholder salience: What happens when the institutional change process unfolds? Journal of Business Ethics, 143(4), 663–680. https://doi.org/10.1007/s10551-015-2766-2</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>What We Know: salience attributes can shift as institutional logic shifts. Supports mid-incident C2 probes.</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>Study design (this is not an institutional-change case of microfinance); theme titles</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
+      <c r="I60" s="6" t="inlineStr">
         <is>
           <t>Wk10 PDF Investigating the Dynamics of Stakeholder Salience</t>
         </is>
       </c>
-      <c r="J53" s="6" t="inlineStr">
+      <c r="J60" s="6" t="inlineStr">
         <is>
           <t>ITDR-GQI-INT-v0.1.1</t>
         </is>
       </c>
-      <c r="K53" s="6" t="inlineStr">
+      <c r="K60" s="6" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="L53" s="6" t="inlineStr">
+      <c r="L60" s="6" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="M53" s="6" t="inlineStr">
+      <c r="M60" s="6" t="inlineStr">
         <is>
           <t>Course PDF. Dynamics claim already implied by C2; do not import the Pakistan microfinance field as this study’s site.</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="48" customHeight="1">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="61" ht="48" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>REF-EMR-ROADMAP-2023</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>seminal_method</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C61" s="6" t="inlineStr">
         <is>
           <t>build_on</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D61" s="6" t="inlineStr">
         <is>
           <t>verify</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E61" s="6" t="inlineStr">
         <is>
           <t>Editorial. (2023). A roadmap for data analysis in qualitative research. European Management Review, 20(2), 190–196. (Duplicate course PDF of the same editorial; authors/page run EM-RAUS230022 — confirm named editorial authors before courseroom paste.)</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>Know Eisenhardt / Gioia / Langley templates so they can be refused as this study’s method</t>
         </is>
       </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="G61" s="6" t="inlineStr">
         <is>
           <t>Declaring Gioia, Eisenhardt, or Langley as the analytic method; replacing Fereday &amp; Muir-Cochrane 2006</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H61" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I54" s="6" t="inlineStr">
+      <c r="I61" s="6" t="inlineStr">
         <is>
           <t>Wk8 duplicate editorials</t>
         </is>
       </c>
-      <c r="J54" s="6" t="inlineStr">
+      <c r="J61" s="6" t="inlineStr">
         <is>
           <t>ITDR-GQI-INT-v0.1.1</t>
         </is>
       </c>
-      <c r="K54" s="6" t="inlineStr">
+      <c r="K61" s="6" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="L54" s="6" t="inlineStr">
+      <c r="L61" s="6" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="M54" s="6" t="inlineStr">
+      <c r="M61" s="6" t="inlineStr">
         <is>
           <t>Two identical PDFs collapsed to one register row. Roadmap is adjacent-method literacy, not a method swap.</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="48" customHeight="1">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="62" ht="48" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>REF-DANIEL-2019</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>comparative</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>build_on</t>
         </is>
       </c>
-      <c r="D55" s="6" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>Daniel, E., &amp; Daniel, P. A. (2019). Megaprojects as complex adaptive systems: The Hinkley Point C case. International Journal of Project Management, 37(8), 1017–1033. https://doi.org/10.1016/j.ijproman.2019.05.001</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F62" s="6" t="inlineStr">
         <is>
           <t>Parking lot / comparative complexity talk only</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G62" s="6" t="inlineStr">
         <is>
           <t>Design; sampling; coding system; Chapter IV themes; replacing GQI</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr">
+      <c r="H62" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I55" s="6" t="inlineStr">
+      <c r="I62" s="6" t="inlineStr">
         <is>
           <t>Wk8 Hinkley Point C PDF</t>
         </is>
       </c>
-      <c r="J55" s="6" t="inlineStr">
+      <c r="J62" s="6" t="inlineStr">
         <is>
           <t>ITDR-GQI-INT-v0.1.1</t>
         </is>
       </c>
-      <c r="K55" s="6" t="inlineStr">
+      <c r="K62" s="6" t="inlineStr">
         <is>
           <t>parked</t>
         </is>
       </c>
-      <c r="L55" s="6" t="inlineStr">
+      <c r="L62" s="6" t="inlineStr">
         <is>
           <t>PARK</t>
         </is>
       </c>
-      <c r="M55" s="6" t="inlineStr">
+      <c r="M62" s="6" t="inlineStr">
         <is>
           <t>Nuclear megaproject CAS is not SME ITDRPaaS GQI. Parked so it cannot leak into method prose.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="48" customHeight="1">
-      <c r="A56" s="6" t="inlineStr">
+    <row r="63" ht="48" customHeight="1">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>REF-CHRISTENSEN-2023</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>comparative</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>build_on</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>Christensen, G. (2024). Three concepts of power: Foucault, Bourdieu, and Habermas. Power and Education, 16(2), 182–195. https://doi.org/10.1177/17577438231187129</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <t>Optional P-memo language only after a concrete force/withhold/override example exists</t>
         </is>
       </c>
-      <c r="G56" s="6" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>Replacing Mitchell power; Delve parent codes; interview stems; educational-theory redesign</t>
         </is>
       </c>
-      <c r="H56" s="6" t="inlineStr">
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I56" s="6" t="inlineStr">
+      <c r="I63" s="6" t="inlineStr">
         <is>
           <t>christensen-2023 PDF</t>
         </is>
       </c>
-      <c r="J56" s="6" t="inlineStr">
+      <c r="J63" s="6" t="inlineStr">
         <is>
           <t>ITDR-GQI-INT-v0.1.1</t>
         </is>
       </c>
-      <c r="K56" s="6" t="inlineStr">
+      <c r="K63" s="6" t="inlineStr">
         <is>
           <t>parked</t>
         </is>
       </c>
-      <c r="L56" s="6" t="inlineStr">
+      <c r="L63" s="6" t="inlineStr">
         <is>
           <t>PARK</t>
         </is>
       </c>
-      <c r="M56" s="6" t="inlineStr">
+      <c r="M63" s="6" t="inlineStr">
         <is>
           <t>Three social-theory powers are not PLU. Parked to stop construct inflation.</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="48" customHeight="1">
-      <c r="A57" s="6" t="inlineStr">
+    <row r="64" ht="48" customHeight="1">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>REF-TRACKING-PACK-2026</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>audit_artifact</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>audit_artifact</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="E57" s="6" t="inlineStr">
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>Walker, M. (2026). Dissertation document tracking pack (Pack v1.0) [Unpublished research operating file]. Capella University, RSCH-V8927. downloads/Dissertation_Document_Tracking_Master.xlsx; downloads/Dissertation_Document_Tracking_Pack.docx.</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <t>Document control; change log; work schedule; folder map</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>Literature source; findings</t>
         </is>
       </c>
-      <c r="H57" s="6" t="inlineStr">
+      <c r="H64" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I57" s="6" t="inlineStr">
+      <c r="I64" s="6" t="inlineStr">
         <is>
           <t>this pack</t>
         </is>
       </c>
-      <c r="J57" s="6" t="inlineStr">
+      <c r="J64" s="6" t="inlineStr">
         <is>
           <t>ITDR-GQI-INT-v0.1.1</t>
         </is>
       </c>
-      <c r="K57" s="6" t="inlineStr">
+      <c r="K64" s="6" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="L57" s="6" t="inlineStr">
+      <c r="L64" s="6" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="M57" s="6" t="inlineStr">
+      <c r="M64" s="6" t="inlineStr">
         <is>
           <t>The consolidated tracker itself is an audit artifact.</t>
         </is>
@@ -8513,12 +8982,12 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>downloads/Dissertation_Document_Tracking_Master.xlsx; downloads/Dissertation_Document_Tracking_Pack.docx; docs/notion/templates/references.csv; docs/notion/templates/update-log.csv</t>
+          <t>downloads/Dissertation_Document_Tracking_Master.xlsx; downloads/Dissertation_Document_Tracking_Pack.docx; docs/notion/templates/references.csv</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Consolidated tracking pack. Spoken wording unchanged. New PDF refs + parking lot. Sample remains 12.</t>
+          <t>Tracking pack v1.0. New PDF refs Joos 2019, Khurram 2015, EMR roadmap 2023, Daniel 2019 parked, Christensen 2023 parked, Wood 2021. Spoken wording unchanged. n=12.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add offering SOP and abstract to success aligned to the tracking pack.
Defines four success outcomes (Need placement, operational PQ answers, inspectable trail, honored gates) and a daily/weekly/stage SOP that reuses locked n=12, instrument v0.1.1, and prior chapter files.

Co-authored-by: delano2x-Procedurals <delano2x-Procedurals@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/Dissertation_Document_Tracking_Master.xlsx
+++ b/downloads/Dissertation_Document_Tracking_Master.xlsx
@@ -24,6 +24,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_PARKING_LOT" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_LEVERAGE_MEMO" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_UPDATE_LOG" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_SOP" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_SUCCESS" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NAVIGATION'!$A$1:$E$1</definedName>
@@ -42,6 +44,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'08_PARKING_LOT'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'11_LEVERAGE_MEMO'!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'12_UPDATE_LOG'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'13_SOP'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'14_SUCCESS'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8705,7 +8709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9001,8 +9005,446 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>UL-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-08T04:40:00Z</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>pack_create</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>researcher</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>docs/offering-sop-and-success-abstract.md; downloads/WALKER_Offering_SOP_and_Success_Abstract.docx; downloads/Dissertation_Document_Tracking_Master.xlsx</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Offering SOP and abstract to success aligned to Need Ch III instrument v0.1.1 and tracking pack. Spoken wording unchanged.</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>docs/notion/templates</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>cadence</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>artifact</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>stop_rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>SOP-D1</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Three-task plan + writing 20–60 min</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Current 01_LIFECYCLE stage</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>No mid-session edit</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>SOP-D2</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Read one source; fill allowed-use</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>03_REFERENCES</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Parked sources stay parked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>SOP-W1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Change log then lifecycle; confirm n=12 and v0.1.1</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>00_CHANGE_LOG; CH3_CONTROL</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Need markdown wins if Word drifted</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SOP-W2</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Weekly (coding)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Interval backup or no_change</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>docs/notion/interval-backups</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Do not overwrite codebook descriptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>SOP-G1</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>IRB gate</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Consent / de-ID / member-check ready</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>revision packet §7</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>No recruitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>SOP-I1</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Interview day</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Q0 first; skip-rules; CLEAN same day</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>05_INTERVIEW_ITEMS; P##</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>No memory-only session; no codebook words in stems</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>SOP-A1</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>MU lock before EMERGENT; two PQ answers</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>06_ANALYSIS_SOP</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Not Gioia; not analyzed-using-Delve</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>prior_output</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Need placed</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>chapter-i-need-for-the-study.md</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>VCST on Need only; ITM alignment pasted</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>VCST as Delve code or theme title</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Gap operational</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>PQ1 / PQ2 in Need + Ch III</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Two Chapter IV answers</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>One governance theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Trail inspectable</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>notion templates + update-log</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Every change has an ID and log row</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Second live codebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Gates honored</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>CH3_CONTROL; parking lot</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>n=12; v0.1.1; IRB before recruit; parked stays parked</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Origins IQ-01 or n=10–15 reopened</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Offering done (Wk 10)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>tracking pack xlsx + docx</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>One xlsx + one Word show locks, Need OV, schedule, next status</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Treating this SOP as a new study</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9013,13 +9455,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -9472,6 +9914,56 @@
       <c r="E18" s="4" t="inlineStr">
         <is>
           <t>APPEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Offering</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>13_SOP</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Daily/weekly/stage SOP for this offering</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>FOLLOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Offering</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>14_SUCCESS</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Abstract-to-success gates vs prior outputs</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>VIEW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close weekly SOP run and refresh tracking documents.
Record UL-0007 no_change, map QUAL headings, and rebuild the master workbook and Word pack so the six weekly todos stay inspectable without changing the spoken protocol or n=12.

Co-authored-by: delano2x-Procedurals <delano2x-Procedurals@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/Dissertation_Document_Tracking_Master.xlsx
+++ b/downloads/Dissertation_Document_Tracking_Master.xlsx
@@ -26,6 +26,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_UPDATE_LOG" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_SOP" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_SUCCESS" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_WEEKLY_RUN" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_QUAL_MAP" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NAVIGATION'!$A$1:$E$1</definedName>
@@ -46,6 +48,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'12_UPDATE_LOG'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'13_SOP'!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'14_SUCCESS'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'15_WEEKLY_RUN'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'16_QUAL_MAP'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8709,7 +8713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9049,6 +9053,53 @@
       <c r="I7" s="5" t="inlineStr">
         <is>
           <t>docs/notion/templates</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>UL-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-08T05:10:00Z</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>no_change</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>ITDR-GQI-INT-v0.1.1</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>researcher</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>docs/weekly-sop-run-2026-09-08.md; docs/notion/interval-backups/2026-09-08-weekly/; downloads/WALKER_Weekly_SOP_Run_2026-09-08.docx</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Weekly SOP §3.3 close. Coding not started so nest copied as no_change. CH3 locks and Need OV confirmed. Spoken wording unchanged. n=12.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>docs/notion/interval-backups/2026-09-08-weekly</t>
         </is>
       </c>
     </row>
@@ -9455,7 +9506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9967,8 +10018,606 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Offering</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>15_WEEKLY_RUN</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-08 weekly SOP six-todo close</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>VIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Alignment</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>16_QUAL_MAP</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>QUAL Example4-1 headings → lifecycle status</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>UPDATE WEEKLY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>sop_step</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Open 00_CHANGE_LOG then 01_LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>12 prior CL rows plus CL-0013/0014 this close. LC-01–04 active/drafted; LC-05–11 not started.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Confirm CH3_CONTROL n=12 and spoken v0.1.1</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Sample locked n=12 (REPLACE vs Origins 10–15). Spoken protocol ITDR-GQI-INT-v0.1.1. VCST Need only. GQI + CIT + hybrid TA + Delve-as-store.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Confirm 09_NEED_OV matches chapter-i markdown</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>N-01–N-09 match Need / ITM / VCST / PQ1 / PQ2 / unit. N-10 records this confirm. Markdown remains source of paste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Interval backup or no_change</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Coding not started. UL-0007 type=no_change. Folder docs/notion/interval-backups/2026-09-08-weekly/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Share one artifact</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>downloads/WALKER_Weekly_SOP_Run_2026-09-08.docx (Need OV + locks + next three tasks).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Map QUAL Example4-1 headings to status</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>16_QUAL_MAP. Collection/IRB/analysis remain Not started. Need/methods drafted.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>qual_heading</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>lifecycle</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>next_action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Alignment to the Program of Study</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>LC-01 / LC-02</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Drafted / In progress</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Paste Need four paragraphs into courseroom Alignment node; do not stack a second Need set</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Project Problem / Gap</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>LC-01</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Keep gap operational (enactment), not definitional</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Supporting Evidence / Synthesis</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>LC-03</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Add REF-IDs with allowed-use; do not replace Mitchell 1997</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Purpose and Project Questions</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>LC-02</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Official RQ labels may replace PQ1/PQ2 tags; unit of analysis stays locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Definition of Terms</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>LC-02</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Use symbols.csv original vs operational defs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Methodological Approach</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>LC-04</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Keep GQI + CIT + hybrid TA; never “analyzed using Delve”</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Population and Sample</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>LC-04 / LC-06</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Drafted lock / collection not started</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>n = 12; 10–200; no recruit before IRB</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Constructs / Phenomena</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>LC-02</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>P L U probes; Lev not a fourth attribute; VCST off Constructs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Measures or Artifacts</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>LC-04</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Instrument v0.1.1; optional artifact Path A/B/C</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Detailed Procedures / Dependability</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>LC-04</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Revision-packet protocol + member-check + storage SOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Sampling Strategy / Recruitment</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>LC-05 / LC-06</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Hard stop until IRB letter</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Data Collection Process</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>LC-07</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Q0 first; skip-rules; CLEAN same day</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Ethical Considerations</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>LC-05</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Capella IRB package from revision packet §7</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Proposed Data Analysis Plan</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>LC-08 / LC-09</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Not started (method drafted)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>MU lock before EMERGENT; two PQ answers</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>References</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>LC-03</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>03_REFERENCES; parked rows stay parked</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9979,7 +10628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10469,6 +11118,80 @@
       <c r="G13" s="5" t="inlineStr">
         <is>
           <t>07_FOLDER_MAP (do-not-edit row)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>CL-0013</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Weekly SOP run 2026-09-08 executed (six todos). CH3 locks confirmed. Need OV matches chapter-i markdown. Coding not started: type=no_change backup dropped. QUAL Example4-1 headings mapped to lifecycle status.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Offering SOP §3.3 requires a weekly close: change log → lifecycle → locks → Need match → nest or no_change → one shareable artifact → QUAL heading status.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>docs/offering-sop-and-success-abstract.md §3.3</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>15_WEEKLY_RUN; 16_QUAL_MAP; downloads/WALKER_Weekly_SOP_Run_2026-09-08.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>CL-0014</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>KEEP</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Parked items remain parked after weekly review. Codebook parents are still STRUCTURAL / FRAMEWORK_DEDUCTIVE / BOUNDARY / EMERGENT (empty). No Foucault, Gioia, or IQ-01 promotion.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Success outcome 4: gates honored.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>04_CODEBOOK; 08_PARKING_LOT</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>08_PARKING_LOT</t>
         </is>
       </c>
     </row>
@@ -10575,7 +11298,11 @@
           <t>Walker</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Advisor packet not yet accepted (weekly 2026-09-08)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -10765,7 +11492,11 @@
           <t>Walker</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>IRB letter (hard gate)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -10803,7 +11534,11 @@
           <t>Walker</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>IRB letter (hard gate)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -11288,7 +12023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11514,6 +12249,28 @@
       <c r="D10" s="4" t="inlineStr">
         <is>
           <t>One U.S. SME IT/network/systems/infrastructure/operations manager; one named disruption, failover, test, or operational recovery in 36 months using external/managed recovery; firm 10–200 personnel; n = 12; interviews only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>N-10</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Weekly Need confirm (2026-09-08)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed matches markdown</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>09_NEED_OV N-01–N-09 agree with docs/chapter-i-need-for-the-study.md: ITM specialization; VCST on Need only; Mitchell PLU on Constructs; implied PQ1/PQ2; interviews-only GQI. Markdown wins if Word drifts.</t>
         </is>
       </c>
     </row>
@@ -11718,17 +12475,17 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>01_LIFECYCLE status; 10_WORK_SCHEDULE checkboxes</t>
+          <t>01_LIFECYCLE status; 15_WEEKLY_RUN; 16_QUAL_MAP</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Pages/sections vs plan; n of sources added</t>
+          <t>Six SOP todos closed; pages/sections vs plan</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Workflow weekly review</t>
+          <t>Workflow weekly review; offering SOP §3.3</t>
         </is>
       </c>
     </row>

</xml_diff>